<commit_message>
Add Superior logo to spreadsheet header
</commit_message>
<xml_diff>
--- a/2026_Safety_Alert_CLEANED.xlsx
+++ b/2026_Safety_Alert_CLEANED.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incident Log'!$A$1:$O$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incident Log'!$A$3:$O$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,16 @@
       <color rgb="001e293b"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001e293b"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f59e0b"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -109,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,6 +137,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -211,6 +223,66 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="523875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -502,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -523,241 +595,113 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>SUPERIOR HUNTINGDON COMPOSITES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>2026 SAFETY ALERT LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Superior/KSS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>Hire Date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>Time of Service</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>Incident Type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>Body Area</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>Corrective Action</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr">
         <is>
           <t>Completed Date</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N3" s="1" t="inlineStr">
         <is>
           <t>Days Away?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O3" s="1" t="inlineStr">
         <is>
           <t>Recordable?</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>1.7.26</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>D team oven</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Jace Ruggles</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>8.14.25</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>approx. 5 months</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Near Miss</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Unrolling mat-mat was sticking together and when pulled back hand was hit by bar</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>left index finger</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>8D form must be completed by forming team. Disciplinary action required</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>Sent email 1/22/26 to see if completed if not, when is it expected to be completed. Sent email 2/3/26 to see if Roger has completed his time on the oven. Alex completed his training on 1.23.26. Roger completed his training on 2.12.26</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>2.12.26</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>1.8.26</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>F team oven</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Aaron Smith</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>5.22.23</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2 yrs 6mo 2wks</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Loss time</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>while gauging the crush roller it was in motion and the roller was tacky and pulled the gauge into th rollers and Aaron's hand was pulled into the roller which was closed at the time allowing his hand to get caught between the top and bottom rollers.</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>left hand</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">oven to be stopped while gauging crush roller. E-stop installed at crush roller. Installing automated crush roller gauge. JSA to be updated to include gauging crush rollers. </t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>sent email 1/22/26 to see if completed with oven associates if not, when is it expected to be completed.</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1.23.26</t>
+          <t>1.7.26</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1st post oven</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Nashika McLean</t>
+          <t>Jace Ruggles</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -767,12 +711,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>6.16.26</t>
+          <t>8.14.25</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>7 months 1 wk</t>
+          <t>approx. 5 months</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -782,27 +726,27 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Turned back from parking dolly and tripped over it and fell</t>
+          <t>Unrolling mat-mat was sticking together and when pulled back hand was hit by bar</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>right elbow &amp; right knee</t>
+          <t>left index finger</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Slow down and take your time, be more observant of your surroundings</t>
+          <t>8D form must be completed by forming team. Disciplinary action required</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Counseled Nashika before returning to the floor. This was discussed with daily safety talks the next work shift.</t>
+          <t>Sent email 1/22/26 to see if completed if not, when is it expected to be completed. Sent email 2/3/26 to see if Roger has completed his time on the oven. Alex completed his training on 1.23.26. Roger completed his training on 2.12.26</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>1.23.26</t>
+          <t>2.12.26</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
@@ -814,21 +758,21 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1.29.26</t>
+          <t>1.8.26</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Parking Lot</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Josh Lister</t>
+          <t>Aaron Smith</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -838,68 +782,68 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>6.30.25</t>
+          <t>5.22.23</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>6 months</t>
+          <t>2 yrs 6mo 2wks</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Near Miss</t>
+          <t>Loss time</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Slipped on ice in parking lot and fell on hip and side.</t>
+          <t>while gauging the crush roller it was in motion and the roller was tacky and pulled the gauge into th rollers and Aaron's hand was pulled into the roller which was closed at the time allowing his hand to get caught between the top and bottom rollers.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>back</t>
+          <t>left hand</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Parking lot was grated after snow fall</t>
+          <t xml:space="preserve">oven to be stopped while gauging crush roller. E-stop installed at crush roller. Installing automated crush roller gauge. JSA to be updated to include gauging crush rollers. </t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Gravel was delivered and spread on 1.30.26</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>1.30.26</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr"/>
+          <t>sent email 1/22/26 to see if completed with oven associates if not, when is it expected to be completed.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2.5.26</t>
+          <t>1.23.26</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>C team forming</t>
+          <t>1st post oven</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Dustin Martin</t>
+          <t>Nashika McLean</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -909,12 +853,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>10.26.23</t>
+          <t>6.16.26</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2 yrs. 3 mo 1 wk</t>
+          <t>7 months 1 wk</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -924,21 +868,29 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>putting fibers on drum and hit right hand on drum slot cutting thumb</t>
+          <t>Turned back from parking dolly and tripped over it and fell</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>right thumb</t>
+          <t>right elbow &amp; right knee</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>No unsafe work practices</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="2" t="n"/>
+          <t>Slow down and take your time, be more observant of your surroundings</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Counseled Nashika before returning to the floor. This was discussed with daily safety talks the next work shift.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>1.23.26</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -948,21 +900,21 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2.15.26</t>
+          <t>1.29.26</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>A team forming</t>
+          <t>Parking Lot</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Kenny Switzer</t>
+          <t>Josh Lister</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -972,12 +924,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>11.10.25</t>
+          <t>6.30.25</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>3 mo 5 days</t>
+          <t>6 months</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -987,25 +939,29 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>While pushing cart from under the drum his strained groin area</t>
+          <t>Slipped on ice in parking lot and fell on hip and side.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>groin</t>
+          <t>back</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>soles of boots are worn bad</t>
+          <t>Parking lot was grated after snow fall</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>placed order for new boots EDT 2.17.26</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="n"/>
+          <t>Gravel was delivered and spread on 1.30.26</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>1.30.26</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -1015,11 +971,11 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>3.8.26</t>
+          <t>2.5.26</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1029,22 +985,22 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Ben Hamm</t>
+          <t>Dustin Martin</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1.12.26</t>
+          <t>10.26.23</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>approx. 2 mo</t>
+          <t>2 yrs. 3 mo 1 wk</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -1054,24 +1010,20 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>pushing out the cart @ unit 39 and lost footage and hit the ground hitting right knee on ground</t>
+          <t>putting fibers on drum and hit right hand on drum slot cutting thumb</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>right knee</t>
+          <t>right thumb</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>check soles of boots</t>
-        </is>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>emailed Danny to check soles of his shoes-- no reply from Danny as of 3.12.26</t>
-        </is>
-      </c>
+          <t>No unsafe work practices</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="n"/>
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="2" t="inlineStr">
@@ -1082,21 +1034,21 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>3.9.26</t>
+          <t>2.15.26</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>A team forming</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Martha Harness</t>
+          <t>Kenny Switzer</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1106,12 +1058,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>12.20.21</t>
+          <t>11.10.25</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>4 yrs. 2.5 mo</t>
+          <t>3 mo 5 days</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1121,22 +1073,22 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Came through the small door and hit her knees on the pull cart that was setting there</t>
+          <t>While pushing cart from under the drum his strained groin area</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>knees</t>
+          <t>groin</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>pull cart was setting there</t>
+          <t>soles of boots are worn bad</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>investigation in progress</t>
+          <t>placed order for new boots EDT 2.17.26</t>
         </is>
       </c>
       <c r="M9" s="2" t="n"/>
@@ -1149,36 +1101,36 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>3.10.26</t>
+          <t>3.8.26</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>C team forming</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Soham Thatte</t>
+          <t>Ben Hamm</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>KSS</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>9.7.21</t>
+          <t>1.12.26</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>4yrs 6 mo 3 days</t>
+          <t>approx. 2 mo</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1188,22 +1140,22 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>bent over looking at pit water level raised back up turned around walking into the corner of the carriage that was setting there</t>
+          <t>pushing out the cart @ unit 39 and lost footage and hit the ground hitting right knee on ground</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>forehead and tooth</t>
+          <t>right knee</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>lack of at tentativeness</t>
+          <t>check soles of boots</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>investigation in progress</t>
+          <t>emailed Danny to check soles of his shoes-- no reply from Danny as of 3.12.26</t>
         </is>
       </c>
       <c r="M10" s="2" t="n"/>
@@ -1216,11 +1168,11 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>3.11.26</t>
+          <t>3.9.26</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1230,7 +1182,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Jace Ruggles</t>
+          <t>Martha Harness</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1240,12 +1192,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>8.14.25</t>
+          <t>12.20.21</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>6 mo 3.5 wks</t>
+          <t>4 yrs. 2.5 mo</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1255,25 +1207,25 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Placing paper in baler and felt something enter his right eye</t>
+          <t>Came through the small door and hit her knees on the pull cart that was setting there</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>right eye</t>
+          <t>knees</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>No unsafe work practices</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>3.11.26</t>
-        </is>
-      </c>
+          <t>pull cart was setting there</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>investigation in progress</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1283,36 +1235,36 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>3.12.26</t>
+          <t>3.10.26</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>F team oven</t>
+          <t>Office</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Alex Unger</t>
+          <t>Soham Thatte</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>3.10.26</t>
+          <t>9.7.21</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>4yrs 6 mo 3 days</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1322,12 +1274,12 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>looking at the ticket on the bar raised head up hitting the keyboard holder</t>
+          <t>bent over looking at pit water level raised back up turned around walking into the corner of the carriage that was setting there</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>forehead</t>
+          <t>forehead and tooth</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -1337,14 +1289,10 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>placed pool noodle around holder. Counseled employee to be more at tentative</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>3.12.26</t>
-        </is>
-      </c>
+          <t>investigation in progress</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1354,11 +1302,11 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>4.13.26</t>
+          <t>3.11.26</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1368,22 +1316,22 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Chris Parker</t>
+          <t>Jace Ruggles</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2.5.26</t>
+          <t>8.14.25</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2 mo 8 days</t>
+          <t>6 mo 3.5 wks</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1393,27 +1341,23 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>while pulling rope through rollers his right shoulder struck against glued mandrel ripping his shirt off</t>
+          <t>Placing paper in baler and felt something enter his right eye</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>right shoulder</t>
+          <t>right eye</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>operator had windup down to close to cutter</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">operator is to keep windup at comfortable distance and not move while pulling rope through oven. </t>
-        </is>
-      </c>
+          <t>No unsafe work practices</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="n"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>4.20.26</t>
+          <t>3.11.26</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr"/>
@@ -1425,21 +1369,21 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4.22.26</t>
+          <t>3.12.26</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Chris Parker</t>
+          <t>Alex Unger</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1449,12 +1393,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2.5.26</t>
+          <t>3.10.26</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2 mo 17 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1464,27 +1408,27 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>placing mandrel in cup when partner shoved bar causing his left ring finger nail to be pinched</t>
+          <t>looking at the ticket on the bar raised head up hitting the keyboard holder</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>left ring finger nail</t>
+          <t>forehead</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>operator instructed his partner to speed up</t>
+          <t>lack of at tentativeness</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>don't rush, work safely</t>
+          <t>placed pool noodle around holder. Counseled employee to be more at tentative</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>4.22.26</t>
+          <t>3.12.26</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr"/>
@@ -1496,84 +1440,92 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>5.5.26</t>
+          <t>4.13.26</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>C team forming</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Breanna Pauley</t>
+          <t>Chris Parker</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>KSS</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>12.15.25</t>
+          <t>2.5.26</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>4 mo 2 wks 5 days</t>
+          <t>2 mo 8 days</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Recordable</t>
+          <t>Near Miss</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>filling dino when glass entered her left eye</t>
+          <t>while pulling rope through rollers his right shoulder struck against glued mandrel ripping his shirt off</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>left eye</t>
+          <t>right shoulder</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>performing normal job duties</t>
-        </is>
-      </c>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="2" t="n"/>
+          <t>operator had windup down to close to cutter</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">operator is to keep windup at comfortable distance and not move while pulling rope through oven. </t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>4.20.26</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>5.5.26</t>
+          <t>4.22.26</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>F team oven</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Jerry Bobbitt</t>
+          <t>Chris Parker</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1583,42 +1535,42 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>4.20.26</t>
+          <t>2.5.26</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>15 days</t>
+          <t>2 mo 17 days</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>near miss</t>
+          <t>Near Miss</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>while pulling rope through the rollers it broke causing left hand to hit bar causing a scratch</t>
+          <t>placing mandrel in cup when partner shoved bar causing his left ring finger nail to be pinched</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>left knuckle</t>
+          <t>left ring finger nail</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>performing normal job duties</t>
+          <t>operator instructed his partner to speed up</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>counseled employees no rushing, work with purpose but not to rush</t>
+          <t>don't rush, work safely</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>5.6.26</t>
+          <t>4.22.26</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
@@ -1630,56 +1582,56 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>6.12.26</t>
+          <t>5.5.26</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>C team forming</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Latoya Thomas</t>
+          <t>Breanna Pauley</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>5.11.26</t>
+          <t>12.15.25</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>1 mo</t>
+          <t>4 mo 2 wks 5 days</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>near miss</t>
+          <t>Recordable</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>putting staples in staple gun-- staple punctured left middle finger</t>
+          <t>filling dino when glass entered her left eye</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>left middle finger</t>
+          <t>left eye</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>lack of at tentativeness</t>
+          <t>performing normal job duties</t>
         </is>
       </c>
       <c r="L17" s="3" t="n"/>
@@ -1687,27 +1639,27 @@
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>6.15.26</t>
+          <t>5.5.26</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Ava Ledford</t>
+          <t>Jerry Bobbitt</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1717,12 +1669,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>6.4.26</t>
+          <t>4.20.26</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>1 wk 4 days</t>
+          <t>15 days</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1732,27 +1684,27 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>right wrist got caught between bar and table belt</t>
+          <t>while pulling rope through the rollers it broke causing left hand to hit bar causing a scratch</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>right wrist</t>
+          <t>left knuckle</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>make sure insert bar is always sticking out of bar to keep mat held back</t>
+          <t>performing normal job duties</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>counseled employee to always make sure insert bar is always sticking out of bar to keep mat held back</t>
+          <t>counseled employees no rushing, work with purpose but not to rush</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>6.15.26</t>
+          <t>5.6.26</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
@@ -1764,21 +1716,21 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>6.29.26</t>
+          <t>6.12.26</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>F team oven</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Jerry Bobbitt</t>
+          <t>Latoya Thomas</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1788,12 +1740,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>4.20.26</t>
+          <t>5.11.26</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2 mo.  9 days</t>
+          <t>1 mo</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1803,25 +1755,21 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>removing bar from roll when finger got pinched between bar and core</t>
+          <t>putting staples in staple gun-- staple punctured left middle finger</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>right ring finger</t>
+          <t>left middle finger</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>no unsafe work practices</t>
+          <t>lack of at tentativeness</t>
         </is>
       </c>
       <c r="L19" s="3" t="n"/>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>6.29.26</t>
-        </is>
-      </c>
+      <c r="M19" s="2" t="n"/>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1831,11 +1779,11 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>8.17.26</t>
+          <t>6.15.26</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1845,22 +1793,22 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Namron Horsley</t>
+          <t>Ava Ledford</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>KSS</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2.27.25</t>
+          <t>6.4.26</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>1 yr. 6 mo.</t>
+          <t>1 wk 4 days</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1870,27 +1818,27 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>slipped and hit head on bar on scale</t>
+          <t>right wrist got caught between bar and table belt</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>right wrist</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>wet floor from AC unit</t>
+          <t>make sure insert bar is always sticking out of bar to keep mat held back</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>make sure AC unit water emptied regularly</t>
+          <t>counseled employee to always make sure insert bar is always sticking out of bar to keep mat held back</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>8.17.26</t>
+          <t>6.15.26</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
@@ -1902,36 +1850,36 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>9.2.26</t>
+          <t>6.29.26</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Post Oven</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Amanda Owens</t>
+          <t>Jerry Bobbitt</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>KSS</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>7.14.26</t>
+          <t>4.20.26</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>1 yr 2 mo.</t>
+          <t>2 mo.  9 days</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1941,25 +1889,25 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>went to grab the bar, mandrel smashed fingers against scale</t>
+          <t>removing bar from roll when finger got pinched between bar and core</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>right middle &amp; ring finger</t>
+          <t>right ring finger</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Partner moving too quickly</t>
-        </is>
-      </c>
-      <c r="L21" s="3" t="inlineStr">
-        <is>
-          <t>reiterate teamwork &amp; communication, have to work together. Implement voice commands "Ready on 1 &amp; ready on 2". Update JSA with voice commands</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n"/>
+          <t>no unsafe work practices</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="n"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>6.29.26</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1969,21 +1917,21 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>9.17.26</t>
+          <t>8.17.26</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Cleanup</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Tommy Ruckel</t>
+          <t>Namron Horsley</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1993,12 +1941,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>4.16.24</t>
+          <t>2.27.25</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2 yrs. 5 mo.</t>
+          <t>1 yr. 6 mo.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -2008,25 +1956,29 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>door grating no positioned properly, when he stepped on it he fell through.</t>
+          <t>slipped and hit head on bar on scale</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>head</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Valicore to ensure they put the grating door back securely after draining pit</t>
+          <t>wet floor from AC unit</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">To email Valicore over incident </t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n"/>
+          <t>make sure AC unit water emptied regularly</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>8.17.26</t>
+        </is>
+      </c>
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -2036,21 +1988,21 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>9.17.26</t>
+          <t>9.2.26</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>Post Oven</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Christina Cooley</t>
+          <t>Amanda Owens</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2060,12 +2012,12 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>10.2.23</t>
+          <t>7.14.26</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2 yrs. 11 mo. 15 days</t>
+          <t>1 yr 2 mo.</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -2075,29 +2027,25 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>She hit her left knee on the motor on her way to shut the buzzer off on the control panel</t>
+          <t>went to grab the bar, mandrel smashed fingers against scale</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>left knee/leg</t>
+          <t>right middle &amp; ring finger</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>unauthorized person shutting belt off</t>
+          <t>Partner moving too quickly</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>disciplinary action taken</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
-        <is>
-          <t>9.17.26</t>
-        </is>
-      </c>
+          <t>reiterate teamwork &amp; communication, have to work together. Implement voice commands "Ready on 1 &amp; ready on 2". Update JSA with voice commands</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n"/>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -2107,103 +2055,103 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>9.24.26</t>
+          <t>9.17.26</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>F team oven</t>
+          <t>Cleanup</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>David Jordan</t>
+          <t>Tommy Ruckel</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>8.21.26</t>
+          <t>4.16.24</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>1 mo. 3 days</t>
+          <t>2 yrs. 5 mo.</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>lost time</t>
+          <t>near miss</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>reach to get hoist &amp; felt sharp pain in stomach (belly button area)</t>
+          <t>door grating no positioned properly, when he stepped on it he fell through.</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>stomach (belly button area)</t>
+          <t>leg</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>possible overexertion or strain</t>
-        </is>
-      </c>
-      <c r="L24" s="3" t="n"/>
+          <t>Valicore to ensure they put the grating door back securely after draining pit</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">To email Valicore over incident </t>
+        </is>
+      </c>
       <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>9.25.26</t>
+          <t>9.17.26</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>C team forming</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Dane Shoemaker</t>
+          <t>Christina Cooley</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>7.9.26</t>
+          <t>10.2.23</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2 mo. 2 wks. 3 days</t>
+          <t>2 yrs. 11 mo. 15 days</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -2213,27 +2161,27 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>pinched skin on right hand with chain of hoist</t>
+          <t>She hit her left knee on the motor on her way to shut the buzzer off on the control panel</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>right hand</t>
+          <t>left knee/leg</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>counseled employee to keep chain tight w/hand</t>
+          <t>unauthorized person shutting belt off</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>wasn't holding cup properly</t>
+          <t>disciplinary action taken</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>9.25.26</t>
+          <t>9.17.26</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr"/>
@@ -2245,87 +2193,226 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>9.24.26</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>F team oven</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>David Jordan</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>8.21.26</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>1 mo. 3 days</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>lost time</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>reach to get hoist &amp; felt sharp pain in stomach (belly button area)</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>stomach (belly button area)</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>possible overexertion or strain</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="n"/>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>9.25.26</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>C team forming</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Dane Shoemaker</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>KSS</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>7.9.26</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2 mo. 2 wks. 3 days</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>near miss</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>pinched skin on right hand with chain of hoist</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>right hand</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>counseled employee to keep chain tight w/hand</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>wasn't holding cup properly</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>9.25.26</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>10.19.26</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>F team oven</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Drake Duncan</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Express</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>10.7.26</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>approx. 3 wks</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>loss time</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>in the process of putting the cup on the bar when his partner raised the hoist and he heard his shoulder pop</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>left shoulder blader</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>not working in sync with his partner</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr">
         <is>
           <t>Include verbal commands in Oven JSA for let off table-- updated JSA on 10.16.26</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>10.21.26</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O26"/>
+  <autoFilter ref="A3:O28"/>
   <conditionalFormatting sqref="O2:O26">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2335,7 +2422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2346,143 +2433,123 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>2026 SAFETY INCIDENT DASHBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>SUPERIOR HUNTINGDON COMPOSITES</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>SUPERIOR HUNTINGDON COMPOSITES</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>2026 SAFETY INCIDENT DASHBOARD</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>YTD TOTAL INCIDENTS</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>RECORDABLES</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>LOSS TIME</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>HAND/FINGER</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>% NEW (&lt;3mo)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="7">
+      <c r="A7" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C7" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G7" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="I5" s="9" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>INCIDENTS BY DEPARTMENT</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>INCIDENTS BY BODY PART</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Body Area</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>D team oven</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>9</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>left index finger</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>F team oven</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>6</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>left hand</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C team forming</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>right elbow &amp; right knee</t>
+          <t>left index finger</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -2492,15 +2559,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1st post oven</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>back</t>
+          <t>left hand</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -2510,15 +2577,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parking Lot</t>
+          <t>C team forming</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>right thumb</t>
+          <t>right elbow &amp; right knee</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -2528,7 +2595,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>A team forming</t>
+          <t>1st post oven</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2536,7 +2603,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>groin</t>
+          <t>back</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -2546,7 +2613,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Parking Lot</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2554,7 +2621,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>right knee</t>
+          <t>right thumb</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -2564,7 +2631,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Post Oven</t>
+          <t>A team forming</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2572,7 +2639,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>knees</t>
+          <t>groin</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -2582,50 +2649,61 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>right knee</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Post Oven</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>knees</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Cleanup</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="inlineStr">
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>forehead and tooth</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="D18" t="inlineStr">
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" t="inlineStr">
         <is>
           <t>right eye</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>forehead</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Data source: 'Incident Log' sheet. Update incidents there — this dashboard auto-counts.</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>right shoulder</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -2635,7 +2713,7 @@
     <row r="21">
       <c r="D21" t="inlineStr">
         <is>
-          <t>left ring finger nail</t>
+          <t>forehead</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -2643,9 +2721,14 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Data source: 'Incident Log' sheet. Update incidents there — this dashboard auto-counts.</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>left eye</t>
+          <t>right shoulder</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -2655,7 +2738,7 @@
     <row r="23">
       <c r="D23" t="inlineStr">
         <is>
-          <t>left knuckle</t>
+          <t>left ring finger nail</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -2665,7 +2748,7 @@
     <row r="24">
       <c r="D24" t="inlineStr">
         <is>
-          <t>left middle finger</t>
+          <t>left eye</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -2675,7 +2758,7 @@
     <row r="25">
       <c r="D25" t="inlineStr">
         <is>
-          <t>right wrist</t>
+          <t>left knuckle</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -2685,7 +2768,7 @@
     <row r="26">
       <c r="D26" t="inlineStr">
         <is>
-          <t>right ring finger</t>
+          <t>left middle finger</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -2695,7 +2778,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>right wrist</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -2705,7 +2788,7 @@
     <row r="28">
       <c r="D28" t="inlineStr">
         <is>
-          <t>right middle &amp; ring finger</t>
+          <t>right ring finger</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -2715,7 +2798,7 @@
     <row r="29">
       <c r="D29" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>head</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2725,7 +2808,7 @@
     <row r="30">
       <c r="D30" t="inlineStr">
         <is>
-          <t>left knee/leg</t>
+          <t>right middle &amp; ring finger</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2735,7 +2818,7 @@
     <row r="31">
       <c r="D31" t="inlineStr">
         <is>
-          <t>stomach (belly button area)</t>
+          <t>leg</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2745,7 +2828,7 @@
     <row r="32">
       <c r="D32" t="inlineStr">
         <is>
-          <t>right hand</t>
+          <t>left knee/leg</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2755,15 +2838,36 @@
     <row r="33">
       <c r="D33" t="inlineStr">
         <is>
+          <t>stomach (belly button area)</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>right hand</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="D35" t="inlineStr">
+        <is>
           <t>left shoulder blader</t>
         </is>
       </c>
-      <c r="E33" t="n">
+      <c r="E35" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix logo layout, no overlap
</commit_message>
<xml_diff>
--- a/2026_Safety_Alert_CLEANED.xlsx
+++ b/2026_Safety_Alert_CLEANED.xlsx
@@ -9,10 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident Log" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incident Log'!$A$3:$O$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incident Log'!$A$4:$O$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,42 +30,18 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="001e293b"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f59e0b"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001e293b"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00f59e0b"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00f59e0b"/>
-      <sz val="28"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00dc2626"/>
-      <sz val="28"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="003b82f6"/>
-      <sz val="28"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001e293b"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -74,12 +49,22 @@
       <sz val="14"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="0064748b"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00f59e0b"/>
-      <sz val="11"/>
+      <sz val="24"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +75,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001e293b"/>
         <bgColor rgb="001e293b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00334155"/>
+        <bgColor rgb="00334155"/>
       </patternFill>
     </fill>
   </fills>
@@ -119,9 +110,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -130,29 +123,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FEE2E2"/>
-          <bgColor rgb="00FEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -234,7 +212,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2095500" cy="571500"/>
+    <ext cx="1905000" cy="523875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -264,7 +242,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="523875"/>
+    <ext cx="1714500" cy="476250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -574,10 +552,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -595,1822 +573,1818 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>SUPERIOR HUNTINGDON COMPOSITES</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>2026 SAFETY ALERT LOG</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2026 Safety Alert Log</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Superior/KSS</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Hire Date</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Time of Service</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Incident Type</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Body Area</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Corrective Action</t>
         </is>
       </c>
-      <c r="L3" s="1" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="M3" s="1" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Completed Date</t>
         </is>
       </c>
-      <c r="N3" s="1" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Days Away?</t>
         </is>
       </c>
-      <c r="O3" s="1" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Recordable?</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+    <row r="5">
+      <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>1.7.26</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Jace Ruggles</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>8.14.25</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>approx. 5 months</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Unrolling mat-mat was sticking together and when pulled back hand was hit by bar</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>left index finger</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>8D form must be completed by forming team. Disciplinary action required</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>Sent email 1/22/26 to see if completed if not, when is it expected to be completed. Sent email 2/3/26 to see if Roger has completed his time on the oven. Alex completed his training on 1.23.26. Roger completed his training on 2.12.26</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>2.12.26</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+    <row r="6">
+      <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>1.8.26</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>F team oven</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Aaron Smith</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>5.22.23</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>2 yrs 6mo 2wks</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Loss time</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>while gauging the crush roller it was in motion and the roller was tacky and pulled the gauge into th rollers and Aaron's hand was pulled into the roller which was closed at the time allowing his hand to get caught between the top and bottom rollers.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>left hand</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">oven to be stopped while gauging crush roller. E-stop installed at crush roller. Installing automated crush roller gauge. JSA to be updated to include gauging crush rollers. </t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>sent email 1/22/26 to see if completed with oven associates if not, when is it expected to be completed.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+    <row r="7">
+      <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>1.23.26</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>1st post oven</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Nashika McLean</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>6.16.26</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>7 months 1 wk</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Turned back from parking dolly and tripped over it and fell</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>right elbow &amp; right knee</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Slow down and take your time, be more observant of your surroundings</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
         <is>
           <t>Counseled Nashika before returning to the floor. This was discussed with daily safety talks the next work shift.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>1.23.26</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr"/>
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+    <row r="8">
+      <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>1.29.26</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Parking Lot</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Josh Lister</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>6.30.25</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>6 months</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Slipped on ice in parking lot and fell on hip and side.</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>back</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Parking lot was grated after snow fall</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>Gravel was delivered and spread on 1.30.26</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>1.30.26</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
+    <row r="9">
+      <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>2.5.26</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>C team forming</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Dustin Martin</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>10.26.23</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>2 yrs. 3 mo 1 wk</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>putting fibers on drum and hit right hand on drum slot cutting thumb</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>right thumb</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>No unsafe work practices</t>
         </is>
       </c>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="inlineStr"/>
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+    <row r="10">
+      <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>2.15.26</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>A team forming</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Kenny Switzer</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>11.10.25</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>3 mo 5 days</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>While pushing cart from under the drum his strained groin area</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>groin</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>soles of boots are worn bad</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>placed order for new boots EDT 2.17.26</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="M10" s="4" t="n"/>
+      <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+    <row r="11">
+      <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>3.8.26</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>C team forming</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Ben Hamm</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>1.12.26</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>approx. 2 mo</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>pushing out the cart @ unit 39 and lost footage and hit the ground hitting right knee on ground</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>right knee</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>check soles of boots</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>emailed Danny to check soles of his shoes-- no reply from Danny as of 3.12.26</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4" t="inlineStr"/>
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+    <row r="12">
+      <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>3.9.26</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Martha Harness</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>12.20.21</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>4 yrs. 2.5 mo</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Came through the small door and hit her knees on the pull cart that was setting there</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>knees</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>pull cart was setting there</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>investigation in progress</t>
         </is>
       </c>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="M12" s="4" t="n"/>
+      <c r="N12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+    <row r="13">
+      <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>3.10.26</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Soham Thatte</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>9.7.21</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>4yrs 6 mo 3 days</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>bent over looking at pit water level raised back up turned around walking into the corner of the carriage that was setting there</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>forehead and tooth</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>lack of at tentativeness</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="L13" s="5" t="inlineStr">
         <is>
           <t>investigation in progress</t>
         </is>
       </c>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="M13" s="4" t="n"/>
+      <c r="N13" s="4" t="inlineStr"/>
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+    <row r="14">
+      <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>3.11.26</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Jace Ruggles</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>8.14.25</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>6 mo 3.5 wks</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Placing paper in baler and felt something enter his right eye</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>right eye</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>No unsafe work practices</t>
         </is>
       </c>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="L14" s="5" t="n"/>
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>3.11.26</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+    <row r="15">
+      <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>3.12.26</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>F team oven</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Alex Unger</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>3.10.26</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>2 days</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>looking at the ticket on the bar raised head up hitting the keyboard holder</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>forehead</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>lack of at tentativeness</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="L15" s="5" t="inlineStr">
         <is>
           <t>placed pool noodle around holder. Counseled employee to be more at tentative</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>3.12.26</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr"/>
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+    <row r="16">
+      <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>4.13.26</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Chris Parker</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>2.5.26</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>2 mo 8 days</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>while pulling rope through rollers his right shoulder struck against glued mandrel ripping his shirt off</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>right shoulder</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>operator had windup down to close to cutter</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">operator is to keep windup at comfortable distance and not move while pulling rope through oven. </t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>4.20.26</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>4.22.26</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Chris Parker</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>2.5.26</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>2 mo 17 days</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>Near Miss</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>placing mandrel in cup when partner shoved bar causing his left ring finger nail to be pinched</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>left ring finger nail</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>operator instructed his partner to speed up</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr">
         <is>
           <t>don't rush, work safely</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>4.22.26</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr"/>
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>5.5.26</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>C team forming</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Breanna Pauley</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>12.15.25</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>4 mo 2 wks 5 days</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>Recordable</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>filling dino when glass entered her left eye</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>left eye</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>performing normal job duties</t>
         </is>
       </c>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="inlineStr"/>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="L18" s="5" t="n"/>
+      <c r="M18" s="4" t="n"/>
+      <c r="N18" s="4" t="inlineStr"/>
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
+    <row r="19">
+      <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>5.5.26</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>F team oven</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Jerry Bobbitt</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>4.20.26</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>15 days</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>while pulling rope through the rollers it broke causing left hand to hit bar causing a scratch</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>left knuckle</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>performing normal job duties</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="L19" s="5" t="inlineStr">
         <is>
           <t>counseled employees no rushing, work with purpose but not to rush</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>5.6.26</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="N19" s="4" t="inlineStr"/>
+      <c r="O19" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
+    <row r="20">
+      <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>6.12.26</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Latoya Thomas</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>5.11.26</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>1 mo</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>putting staples in staple gun-- staple punctured left middle finger</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>left middle finger</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>lack of at tentativeness</t>
         </is>
       </c>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="L20" s="5" t="n"/>
+      <c r="M20" s="4" t="n"/>
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
+    <row r="21">
+      <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>6.15.26</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Ava Ledford</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>6.4.26</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>1 wk 4 days</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>right wrist got caught between bar and table belt</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>right wrist</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>make sure insert bar is always sticking out of bar to keep mat held back</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="L21" s="5" t="inlineStr">
         <is>
           <t>counseled employee to always make sure insert bar is always sticking out of bar to keep mat held back</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>6.15.26</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr"/>
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
+    <row r="22">
+      <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>6.29.26</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>F team oven</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Jerry Bobbitt</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>4.20.26</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>2 mo.  9 days</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>removing bar from roll when finger got pinched between bar and core</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>right ring finger</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>no unsafe work practices</t>
         </is>
       </c>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="L22" s="5" t="n"/>
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>6.29.26</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr"/>
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
+    <row r="23">
+      <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>8.17.26</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Namron Horsley</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>2.27.25</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>1 yr. 6 mo.</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>slipped and hit head on bar on scale</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>head</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>wet floor from AC unit</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
         <is>
           <t>make sure AC unit water emptied regularly</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>8.17.26</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr"/>
+      <c r="O23" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
+    <row r="24">
+      <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>9.2.26</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Post Oven</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Amanda Owens</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>7.14.26</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>1 yr 2 mo.</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>went to grab the bar, mandrel smashed fingers against scale</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>right middle &amp; ring finger</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
         <is>
           <t>Partner moving too quickly</t>
         </is>
       </c>
-      <c r="L23" s="3" t="inlineStr">
+      <c r="L24" s="5" t="inlineStr">
         <is>
           <t>reiterate teamwork &amp; communication, have to work together. Implement voice commands "Ready on 1 &amp; ready on 2". Update JSA with voice commands</t>
         </is>
       </c>
-      <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="M24" s="4" t="n"/>
+      <c r="N24" s="4" t="inlineStr"/>
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
+    <row r="25">
+      <c r="A25" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>9.17.26</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Tommy Ruckel</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>4.16.24</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>2 yrs. 5 mo.</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>door grating no positioned properly, when he stepped on it he fell through.</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>leg</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K25" s="5" t="inlineStr">
         <is>
           <t>Valicore to ensure they put the grating door back securely after draining pit</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="L25" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">To email Valicore over incident </t>
         </is>
       </c>
-      <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4" t="inlineStr"/>
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
+    <row r="26">
+      <c r="A26" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>9.17.26</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>D team oven</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Christina Cooley</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Superior</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>10.2.23</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>2 yrs. 11 mo. 15 days</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>She hit her left knee on the motor on her way to shut the buzzer off on the control panel</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>left knee/leg</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K26" s="5" t="inlineStr">
         <is>
           <t>unauthorized person shutting belt off</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr">
+      <c r="L26" s="5" t="inlineStr">
         <is>
           <t>disciplinary action taken</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>9.17.26</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr"/>
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
+    <row r="27">
+      <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>9.24.26</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>F team oven</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>David Jordan</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Express</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>8.21.26</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>1 mo. 3 days</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>lost time</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>reach to get hoist &amp; felt sharp pain in stomach (belly button area)</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>stomach (belly button area)</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K27" s="5" t="inlineStr">
         <is>
           <t>possible overexertion or strain</t>
         </is>
       </c>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="2" t="n"/>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="L27" s="5" t="n"/>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
+    <row r="28">
+      <c r="A28" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>9.25.26</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>C team forming</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Dane Shoemaker</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>KSS</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>7.9.26</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>2 mo. 2 wks. 3 days</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>near miss</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>pinched skin on right hand with chain of hoist</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>right hand</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K28" s="5" t="inlineStr">
         <is>
           <t>counseled employee to keep chain tight w/hand</t>
         </is>
       </c>
-      <c r="L27" s="3" t="inlineStr">
+      <c r="L28" s="5" t="inlineStr">
         <is>
           <t>wasn't holding cup properly</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>9.25.26</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr"/>
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
+    <row r="29">
+      <c r="A29" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>10.19.26</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>F team oven</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Drake Duncan</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Express</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>10.7.26</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>approx. 3 wks</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>loss time</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>in the process of putting the cup on the bar when his partner raised the hoist and he heard his shoulder pop</t>
         </is>
       </c>
-      <c r="J28" s="3" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>left shoulder blader</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K29" s="5" t="inlineStr">
         <is>
           <t>not working in sync with his partner</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="L29" s="5" t="inlineStr">
         <is>
           <t>Include verbal commands in Oven JSA for let off table-- updated JSA on 10.16.26</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="M29" s="4" t="inlineStr">
         <is>
           <t>10.21.26</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="O29" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:O28"/>
-  <conditionalFormatting sqref="O2:O26">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"Yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <autoFilter ref="A4:O29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -2422,560 +2396,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>2026 SAFETY INCIDENT DASHBOARD</t>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>2026 Safety Incident Dashboard</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>SUPERIOR HUNTINGDON COMPOSITES</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>SUPERIOR HUNTINGDON COMPOSITES</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>2026 SAFETY INCIDENT DASHBOARD</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Source: Incident Log tab — counts update automatically</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>YTD TOTAL INCIDENTS</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>RECORDABLES</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>LOSS TIME</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>HAND/FINGER</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>YTD TOTAL INCIDENTS</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>RECORDABLES</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>LOSS TIME</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>HAND/FINGER</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>% NEW (&lt;3mo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A6" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="7" t="n">
+      <c r="G6" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="9" t="n">
         <v>10</v>
-      </c>
-      <c r="I7" s="9" t="inlineStr"/>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>INCIDENTS BY DEPARTMENT</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>INCIDENTS BY BODY PART</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Body Area</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>D team oven</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>9</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>left index finger</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>F team oven</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>6</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>left hand</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>C team forming</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>right elbow &amp; right knee</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1st post oven</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>back</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Parking Lot</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>right thumb</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>A team forming</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>groin</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>right knee</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Post Oven</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>knees</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>forehead and tooth</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>right eye</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>forehead</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Data source: 'Incident Log' sheet. Update incidents there — this dashboard auto-counts.</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>right shoulder</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>left ring finger nail</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>left eye</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>left knuckle</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>left middle finger</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>right wrist</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>right ring finger</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>right middle &amp; ring finger</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>leg</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>left knee/leg</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>stomach (belly button area)</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>right hand</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>left shoulder blader</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Departments</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Incident Types</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1st post oven</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Near Miss</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>A team forming</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Recordable</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>C team forming</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Loss Time</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Lost Time</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>D team oven</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>F team oven</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Office</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Parking Lot</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Post Oven</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Stacked header, no gap column
</commit_message>
<xml_diff>
--- a/2026_Safety_Alert_CLEANED.xlsx
+++ b/2026_Safety_Alert_CLEANED.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incident Log'!$A$4:$O$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incident Log'!$A$6:$O$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +31,7 @@
     <font>
       <b val="1"/>
       <color rgb="001e293b"/>
-      <sz val="15"/>
+      <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
@@ -46,7 +46,7 @@
     <font>
       <b val="1"/>
       <color rgb="001e293b"/>
-      <sz val="14"/>
+      <sz val="15"/>
     </font>
     <font>
       <i val="1"/>
@@ -61,7 +61,7 @@
     <font>
       <b val="1"/>
       <color rgb="00f59e0b"/>
-      <sz val="24"/>
+      <sz val="26"/>
     </font>
   </fonts>
   <fills count="4">
@@ -212,7 +212,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="523875"/>
+    <ext cx="1714500" cy="476250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -242,7 +242,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1714500" cy="476250"/>
+    <ext cx="1619250" cy="457200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A3:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -572,257 +572,115 @@
     <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>SUPERIOR HUNTINGDON COMPOSITES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>2026 Safety Alert Log</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>2026 SAFETY ALERT LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Superior Huntingdon Composites</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="10" customHeight="1"/>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Superior/KSS</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Hire Date</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Time of Service</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Incident Type</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Body Area</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>Corrective Action</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>Completed Date</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>Days Away?</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>Recordable?</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>1.7.26</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>D team oven</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Jace Ruggles</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>8.14.25</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>approx. 5 months</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Near Miss</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Unrolling mat-mat was sticking together and when pulled back hand was hit by bar</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>left index finger</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>8D form must be completed by forming team. Disciplinary action required</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Sent email 1/22/26 to see if completed if not, when is it expected to be completed. Sent email 2/3/26 to see if Roger has completed his time on the oven. Alex completed his training on 1.23.26. Roger completed his training on 2.12.26</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>2.12.26</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>1.8.26</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>F team oven</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Aaron Smith</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>5.22.23</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>2 yrs 6mo 2wks</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Loss time</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>while gauging the crush roller it was in motion and the roller was tacky and pulled the gauge into th rollers and Aaron's hand was pulled into the roller which was closed at the time allowing his hand to get caught between the top and bottom rollers.</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>left hand</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">oven to be stopped while gauging crush roller. E-stop installed at crush roller. Installing automated crush roller gauge. JSA to be updated to include gauging crush rollers. </t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>sent email 1/22/26 to see if completed with oven associates if not, when is it expected to be completed.</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="n"/>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>1.23.26</t>
+          <t>1.7.26</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>1st post oven</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Nashika McLean</t>
+          <t>Jace Ruggles</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -832,12 +690,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>6.16.26</t>
+          <t>8.14.25</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>7 months 1 wk</t>
+          <t>approx. 5 months</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -847,27 +705,27 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Turned back from parking dolly and tripped over it and fell</t>
+          <t>Unrolling mat-mat was sticking together and when pulled back hand was hit by bar</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>right elbow &amp; right knee</t>
+          <t>left index finger</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Slow down and take your time, be more observant of your surroundings</t>
+          <t>8D form must be completed by forming team. Disciplinary action required</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Counseled Nashika before returning to the floor. This was discussed with daily safety talks the next work shift.</t>
+          <t>Sent email 1/22/26 to see if completed if not, when is it expected to be completed. Sent email 2/3/26 to see if Roger has completed his time on the oven. Alex completed his training on 1.23.26. Roger completed his training on 2.12.26</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>1.23.26</t>
+          <t>2.12.26</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr"/>
@@ -879,21 +737,21 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>1.29.26</t>
+          <t>1.8.26</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Parking Lot</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Josh Lister</t>
+          <t>Aaron Smith</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -903,68 +761,68 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>6.30.25</t>
+          <t>5.22.23</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>6 months</t>
+          <t>2 yrs 6mo 2wks</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Near Miss</t>
+          <t>Loss time</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Slipped on ice in parking lot and fell on hip and side.</t>
+          <t>while gauging the crush roller it was in motion and the roller was tacky and pulled the gauge into th rollers and Aaron's hand was pulled into the roller which was closed at the time allowing his hand to get caught between the top and bottom rollers.</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>back</t>
+          <t>left hand</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Parking lot was grated after snow fall</t>
+          <t xml:space="preserve">oven to be stopped while gauging crush roller. E-stop installed at crush roller. Installing automated crush roller gauge. JSA to be updated to include gauging crush rollers. </t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Gravel was delivered and spread on 1.30.26</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>1.30.26</t>
-        </is>
-      </c>
-      <c r="N8" s="4" t="inlineStr"/>
+          <t>sent email 1/22/26 to see if completed with oven associates if not, when is it expected to be completed.</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2.5.26</t>
+          <t>1.23.26</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>C team forming</t>
+          <t>1st post oven</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Dustin Martin</t>
+          <t>Nashika McLean</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -974,12 +832,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>10.26.23</t>
+          <t>6.16.26</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2 yrs. 3 mo 1 wk</t>
+          <t>7 months 1 wk</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -989,21 +847,29 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>putting fibers on drum and hit right hand on drum slot cutting thumb</t>
+          <t>Turned back from parking dolly and tripped over it and fell</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>right thumb</t>
+          <t>right elbow &amp; right knee</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>No unsafe work practices</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="4" t="n"/>
+          <t>Slow down and take your time, be more observant of your surroundings</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Counseled Nashika before returning to the floor. This was discussed with daily safety talks the next work shift.</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>1.23.26</t>
+        </is>
+      </c>
       <c r="N9" s="4" t="inlineStr"/>
       <c r="O9" s="4" t="inlineStr">
         <is>
@@ -1013,21 +879,21 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>2.15.26</t>
+          <t>1.29.26</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>A team forming</t>
+          <t>Parking Lot</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Kenny Switzer</t>
+          <t>Josh Lister</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1037,12 +903,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>11.10.25</t>
+          <t>6.30.25</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>3 mo 5 days</t>
+          <t>6 months</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1052,25 +918,29 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>While pushing cart from under the drum his strained groin area</t>
+          <t>Slipped on ice in parking lot and fell on hip and side.</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>groin</t>
+          <t>back</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>soles of boots are worn bad</t>
+          <t>Parking lot was grated after snow fall</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>placed order for new boots EDT 2.17.26</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="n"/>
+          <t>Gravel was delivered and spread on 1.30.26</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>1.30.26</t>
+        </is>
+      </c>
       <c r="N10" s="4" t="inlineStr"/>
       <c r="O10" s="4" t="inlineStr">
         <is>
@@ -1080,11 +950,11 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>3.8.26</t>
+          <t>2.5.26</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1094,22 +964,22 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Ben Hamm</t>
+          <t>Dustin Martin</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>1.12.26</t>
+          <t>10.26.23</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>approx. 2 mo</t>
+          <t>2 yrs. 3 mo 1 wk</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1119,24 +989,20 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>pushing out the cart @ unit 39 and lost footage and hit the ground hitting right knee on ground</t>
+          <t>putting fibers on drum and hit right hand on drum slot cutting thumb</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>right knee</t>
+          <t>right thumb</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>check soles of boots</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>emailed Danny to check soles of his shoes-- no reply from Danny as of 3.12.26</t>
-        </is>
-      </c>
+          <t>No unsafe work practices</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="n"/>
       <c r="M11" s="4" t="n"/>
       <c r="N11" s="4" t="inlineStr"/>
       <c r="O11" s="4" t="inlineStr">
@@ -1147,21 +1013,21 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>3.9.26</t>
+          <t>2.15.26</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>A team forming</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Martha Harness</t>
+          <t>Kenny Switzer</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1171,12 +1037,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>12.20.21</t>
+          <t>11.10.25</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>4 yrs. 2.5 mo</t>
+          <t>3 mo 5 days</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1186,22 +1052,22 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Came through the small door and hit her knees on the pull cart that was setting there</t>
+          <t>While pushing cart from under the drum his strained groin area</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>knees</t>
+          <t>groin</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>pull cart was setting there</t>
+          <t>soles of boots are worn bad</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>investigation in progress</t>
+          <t>placed order for new boots EDT 2.17.26</t>
         </is>
       </c>
       <c r="M12" s="4" t="n"/>
@@ -1214,36 +1080,36 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>3.10.26</t>
+          <t>3.8.26</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>C team forming</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Soham Thatte</t>
+          <t>Ben Hamm</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>KSS</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>9.7.21</t>
+          <t>1.12.26</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>4yrs 6 mo 3 days</t>
+          <t>approx. 2 mo</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1253,22 +1119,22 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>bent over looking at pit water level raised back up turned around walking into the corner of the carriage that was setting there</t>
+          <t>pushing out the cart @ unit 39 and lost footage and hit the ground hitting right knee on ground</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>forehead and tooth</t>
+          <t>right knee</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>lack of at tentativeness</t>
+          <t>check soles of boots</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>investigation in progress</t>
+          <t>emailed Danny to check soles of his shoes-- no reply from Danny as of 3.12.26</t>
         </is>
       </c>
       <c r="M13" s="4" t="n"/>
@@ -1281,11 +1147,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>3.11.26</t>
+          <t>3.9.26</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1295,7 +1161,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Jace Ruggles</t>
+          <t>Martha Harness</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1305,12 +1171,12 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>8.14.25</t>
+          <t>12.20.21</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>6 mo 3.5 wks</t>
+          <t>4 yrs. 2.5 mo</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1320,25 +1186,25 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Placing paper in baler and felt something enter his right eye</t>
+          <t>Came through the small door and hit her knees on the pull cart that was setting there</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>right eye</t>
+          <t>knees</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>No unsafe work practices</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>3.11.26</t>
-        </is>
-      </c>
+          <t>pull cart was setting there</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>investigation in progress</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="n"/>
       <c r="N14" s="4" t="inlineStr"/>
       <c r="O14" s="4" t="inlineStr">
         <is>
@@ -1348,36 +1214,36 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>3.12.26</t>
+          <t>3.10.26</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>F team oven</t>
+          <t>Office</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Alex Unger</t>
+          <t>Soham Thatte</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>3.10.26</t>
+          <t>9.7.21</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>4yrs 6 mo 3 days</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1387,12 +1253,12 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>looking at the ticket on the bar raised head up hitting the keyboard holder</t>
+          <t>bent over looking at pit water level raised back up turned around walking into the corner of the carriage that was setting there</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>forehead</t>
+          <t>forehead and tooth</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -1402,14 +1268,10 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>placed pool noodle around holder. Counseled employee to be more at tentative</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>3.12.26</t>
-        </is>
-      </c>
+          <t>investigation in progress</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="n"/>
       <c r="N15" s="4" t="inlineStr"/>
       <c r="O15" s="4" t="inlineStr">
         <is>
@@ -1419,11 +1281,11 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>4.13.26</t>
+          <t>3.11.26</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1433,22 +1295,22 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Chris Parker</t>
+          <t>Jace Ruggles</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>2.5.26</t>
+          <t>8.14.25</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>2 mo 8 days</t>
+          <t>6 mo 3.5 wks</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1458,27 +1320,23 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>while pulling rope through rollers his right shoulder struck against glued mandrel ripping his shirt off</t>
+          <t>Placing paper in baler and felt something enter his right eye</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>right shoulder</t>
+          <t>right eye</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>operator had windup down to close to cutter</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">operator is to keep windup at comfortable distance and not move while pulling rope through oven. </t>
-        </is>
-      </c>
+          <t>No unsafe work practices</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="n"/>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>4.20.26</t>
+          <t>3.11.26</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr"/>
@@ -1490,21 +1348,21 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>4.22.26</t>
+          <t>3.12.26</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Chris Parker</t>
+          <t>Alex Unger</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1514,12 +1372,12 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>2.5.26</t>
+          <t>3.10.26</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2 mo 17 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1529,27 +1387,27 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>placing mandrel in cup when partner shoved bar causing his left ring finger nail to be pinched</t>
+          <t>looking at the ticket on the bar raised head up hitting the keyboard holder</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>left ring finger nail</t>
+          <t>forehead</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>operator instructed his partner to speed up</t>
+          <t>lack of at tentativeness</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>don't rush, work safely</t>
+          <t>placed pool noodle around holder. Counseled employee to be more at tentative</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>4.22.26</t>
+          <t>3.12.26</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr"/>
@@ -1561,84 +1419,92 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>5.5.26</t>
+          <t>4.13.26</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>C team forming</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Breanna Pauley</t>
+          <t>Chris Parker</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>KSS</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>12.15.25</t>
+          <t>2.5.26</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>4 mo 2 wks 5 days</t>
+          <t>2 mo 8 days</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Recordable</t>
+          <t>Near Miss</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>filling dino when glass entered her left eye</t>
+          <t>while pulling rope through rollers his right shoulder struck against glued mandrel ripping his shirt off</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>left eye</t>
+          <t>right shoulder</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>performing normal job duties</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="n"/>
-      <c r="M18" s="4" t="n"/>
+          <t>operator had windup down to close to cutter</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">operator is to keep windup at comfortable distance and not move while pulling rope through oven. </t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>4.20.26</t>
+        </is>
+      </c>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>5.5.26</t>
+          <t>4.22.26</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>F team oven</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Jerry Bobbitt</t>
+          <t>Chris Parker</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1648,42 +1514,42 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>4.20.26</t>
+          <t>2.5.26</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>15 days</t>
+          <t>2 mo 17 days</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>near miss</t>
+          <t>Near Miss</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>while pulling rope through the rollers it broke causing left hand to hit bar causing a scratch</t>
+          <t>placing mandrel in cup when partner shoved bar causing his left ring finger nail to be pinched</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>left knuckle</t>
+          <t>left ring finger nail</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>performing normal job duties</t>
+          <t>operator instructed his partner to speed up</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>counseled employees no rushing, work with purpose but not to rush</t>
+          <t>don't rush, work safely</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>5.6.26</t>
+          <t>4.22.26</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr"/>
@@ -1695,56 +1561,56 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>6.12.26</t>
+          <t>5.5.26</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>C team forming</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Latoya Thomas</t>
+          <t>Breanna Pauley</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>5.11.26</t>
+          <t>12.15.25</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>1 mo</t>
+          <t>4 mo 2 wks 5 days</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>near miss</t>
+          <t>Recordable</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>putting staples in staple gun-- staple punctured left middle finger</t>
+          <t>filling dino when glass entered her left eye</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>left middle finger</t>
+          <t>left eye</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>lack of at tentativeness</t>
+          <t>performing normal job duties</t>
         </is>
       </c>
       <c r="L20" s="5" t="n"/>
@@ -1752,27 +1618,27 @@
       <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>6.15.26</t>
+          <t>5.5.26</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Ava Ledford</t>
+          <t>Jerry Bobbitt</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1782,12 +1648,12 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>6.4.26</t>
+          <t>4.20.26</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>1 wk 4 days</t>
+          <t>15 days</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1797,27 +1663,27 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>right wrist got caught between bar and table belt</t>
+          <t>while pulling rope through the rollers it broke causing left hand to hit bar causing a scratch</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>right wrist</t>
+          <t>left knuckle</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>make sure insert bar is always sticking out of bar to keep mat held back</t>
+          <t>performing normal job duties</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>counseled employee to always make sure insert bar is always sticking out of bar to keep mat held back</t>
+          <t>counseled employees no rushing, work with purpose but not to rush</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>6.15.26</t>
+          <t>5.6.26</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr"/>
@@ -1829,21 +1695,21 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>6.29.26</t>
+          <t>6.12.26</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>F team oven</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Jerry Bobbitt</t>
+          <t>Latoya Thomas</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1853,12 +1719,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>4.20.26</t>
+          <t>5.11.26</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>2 mo.  9 days</t>
+          <t>1 mo</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -1868,25 +1734,21 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>removing bar from roll when finger got pinched between bar and core</t>
+          <t>putting staples in staple gun-- staple punctured left middle finger</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>right ring finger</t>
+          <t>left middle finger</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>no unsafe work practices</t>
+          <t>lack of at tentativeness</t>
         </is>
       </c>
       <c r="L22" s="5" t="n"/>
-      <c r="M22" s="4" t="inlineStr">
-        <is>
-          <t>6.29.26</t>
-        </is>
-      </c>
+      <c r="M22" s="4" t="n"/>
       <c r="N22" s="4" t="inlineStr"/>
       <c r="O22" s="4" t="inlineStr">
         <is>
@@ -1896,11 +1758,11 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>8.17.26</t>
+          <t>6.15.26</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1910,22 +1772,22 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Namron Horsley</t>
+          <t>Ava Ledford</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>KSS</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>2.27.25</t>
+          <t>6.4.26</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>1 yr. 6 mo.</t>
+          <t>1 wk 4 days</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1935,27 +1797,27 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>slipped and hit head on bar on scale</t>
+          <t>right wrist got caught between bar and table belt</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>right wrist</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>wet floor from AC unit</t>
+          <t>make sure insert bar is always sticking out of bar to keep mat held back</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>make sure AC unit water emptied regularly</t>
+          <t>counseled employee to always make sure insert bar is always sticking out of bar to keep mat held back</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>8.17.26</t>
+          <t>6.15.26</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr"/>
@@ -1967,36 +1829,36 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>9.2.26</t>
+          <t>6.29.26</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Post Oven</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Amanda Owens</t>
+          <t>Jerry Bobbitt</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>KSS</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>7.14.26</t>
+          <t>4.20.26</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>1 yr 2 mo.</t>
+          <t>2 mo.  9 days</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -2006,25 +1868,25 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>went to grab the bar, mandrel smashed fingers against scale</t>
+          <t>removing bar from roll when finger got pinched between bar and core</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>right middle &amp; ring finger</t>
+          <t>right ring finger</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>Partner moving too quickly</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>reiterate teamwork &amp; communication, have to work together. Implement voice commands "Ready on 1 &amp; ready on 2". Update JSA with voice commands</t>
-        </is>
-      </c>
-      <c r="M24" s="4" t="n"/>
+          <t>no unsafe work practices</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="n"/>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>6.29.26</t>
+        </is>
+      </c>
       <c r="N24" s="4" t="inlineStr"/>
       <c r="O24" s="4" t="inlineStr">
         <is>
@@ -2034,21 +1896,21 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>9.17.26</t>
+          <t>8.17.26</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Cleanup</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Tommy Ruckel</t>
+          <t>Namron Horsley</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2058,12 +1920,12 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>4.16.24</t>
+          <t>2.27.25</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>2 yrs. 5 mo.</t>
+          <t>1 yr. 6 mo.</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -2073,25 +1935,29 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>door grating no positioned properly, when he stepped on it he fell through.</t>
+          <t>slipped and hit head on bar on scale</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>head</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>Valicore to ensure they put the grating door back securely after draining pit</t>
+          <t>wet floor from AC unit</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">To email Valicore over incident </t>
-        </is>
-      </c>
-      <c r="M25" s="4" t="n"/>
+          <t>make sure AC unit water emptied regularly</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>8.17.26</t>
+        </is>
+      </c>
       <c r="N25" s="4" t="inlineStr"/>
       <c r="O25" s="4" t="inlineStr">
         <is>
@@ -2101,21 +1967,21 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>9.17.26</t>
+          <t>9.2.26</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>D team oven</t>
+          <t>Post Oven</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Christina Cooley</t>
+          <t>Amanda Owens</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2125,12 +1991,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>10.2.23</t>
+          <t>7.14.26</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>2 yrs. 11 mo. 15 days</t>
+          <t>1 yr 2 mo.</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -2140,29 +2006,25 @@
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>She hit her left knee on the motor on her way to shut the buzzer off on the control panel</t>
+          <t>went to grab the bar, mandrel smashed fingers against scale</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>left knee/leg</t>
+          <t>right middle &amp; ring finger</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>unauthorized person shutting belt off</t>
+          <t>Partner moving too quickly</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>disciplinary action taken</t>
-        </is>
-      </c>
-      <c r="M26" s="4" t="inlineStr">
-        <is>
-          <t>9.17.26</t>
-        </is>
-      </c>
+          <t>reiterate teamwork &amp; communication, have to work together. Implement voice commands "Ready on 1 &amp; ready on 2". Update JSA with voice commands</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="n"/>
       <c r="N26" s="4" t="inlineStr"/>
       <c r="O26" s="4" t="inlineStr">
         <is>
@@ -2172,103 +2034,103 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>9.24.26</t>
+          <t>9.17.26</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>F team oven</t>
+          <t>Cleanup</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>David Jordan</t>
+          <t>Tommy Ruckel</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>8.21.26</t>
+          <t>4.16.24</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>1 mo. 3 days</t>
+          <t>2 yrs. 5 mo.</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>lost time</t>
+          <t>near miss</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>reach to get hoist &amp; felt sharp pain in stomach (belly button area)</t>
+          <t>door grating no positioned properly, when he stepped on it he fell through.</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>stomach (belly button area)</t>
+          <t>leg</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>possible overexertion or strain</t>
-        </is>
-      </c>
-      <c r="L27" s="5" t="n"/>
+          <t>Valicore to ensure they put the grating door back securely after draining pit</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">To email Valicore over incident </t>
+        </is>
+      </c>
       <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N27" s="4" t="inlineStr"/>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>9.25.26</t>
+          <t>9.17.26</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>C team forming</t>
+          <t>D team oven</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Dane Shoemaker</t>
+          <t>Christina Cooley</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>KSS</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>7.9.26</t>
+          <t>10.2.23</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>2 mo. 2 wks. 3 days</t>
+          <t>2 yrs. 11 mo. 15 days</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2278,27 +2140,27 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>pinched skin on right hand with chain of hoist</t>
+          <t>She hit her left knee on the motor on her way to shut the buzzer off on the control panel</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>right hand</t>
+          <t>left knee/leg</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>counseled employee to keep chain tight w/hand</t>
+          <t>unauthorized person shutting belt off</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>wasn't holding cup properly</t>
+          <t>disciplinary action taken</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>9.25.26</t>
+          <t>9.17.26</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr"/>
@@ -2310,81 +2172,219 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>9.24.26</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>F team oven</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>David Jordan</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>8.21.26</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>1 mo. 3 days</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>lost time</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>reach to get hoist &amp; felt sharp pain in stomach (belly button area)</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>stomach (belly button area)</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>possible overexertion or strain</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="n"/>
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>9.25.26</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>C team forming</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Dane Shoemaker</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>KSS</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>7.9.26</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>2 mo. 2 wks. 3 days</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>near miss</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>pinched skin on right hand with chain of hoist</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>right hand</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>counseled employee to keep chain tight w/hand</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>wasn't holding cup properly</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>9.25.26</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr"/>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>10.19.26</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>F team oven</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Drake Duncan</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>Express</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>10.7.26</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>approx. 3 wks</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>loss time</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>in the process of putting the cup on the bar when his partner raised the hoist and he heard his shoulder pop</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>left shoulder blader</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr">
+      <c r="K31" s="5" t="inlineStr">
         <is>
           <t>not working in sync with his partner</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="L31" s="5" t="inlineStr">
         <is>
           <t>Include verbal commands in Oven JSA for let off table-- updated JSA on 10.16.26</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>10.21.26</t>
         </is>
       </c>
-      <c r="N29" s="4" t="inlineStr">
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O29" s="4" t="inlineStr">
+      <c r="O31" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O29"/>
+  <autoFilter ref="A6:O31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -2396,63 +2396,69 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A3:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>2026 Safety Incident Dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>SUPERIOR HUNTINGDON COMPOSITES</t>
-        </is>
-      </c>
-    </row>
     <row r="3">
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Source: Incident Log tab — counts update automatically</t>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>2026 SAFETY INCIDENT DASHBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Superior Huntingdon Composites</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>YTD TOTAL INCIDENTS</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Counts update automatically from the Incident Log tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>YTD TOTAL</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>RECORDABLES</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>LOSS TIME</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>HAND/FINGER</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="n">
+    <row r="8">
+      <c r="A8" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D8" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="9" t="n">
+      <c r="J8" s="9" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Merged header cells, thin column A
</commit_message>
<xml_diff>
--- a/2026_Safety_Alert_CLEANED.xlsx
+++ b/2026_Safety_Alert_CLEANED.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,11 +47,6 @@
       <b val="1"/>
       <color rgb="001e293b"/>
       <sz val="15"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="0064748b"/>
-      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -110,10 +105,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -123,10 +122,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -212,7 +222,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1714500" cy="476250"/>
+    <ext cx="1809750" cy="495300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -242,7 +252,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1619250" cy="457200"/>
+    <ext cx="1619250" cy="447675"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -552,10 +562,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:O31"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -572,21 +582,23 @@
     <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="3">
+    <row r="1" ht="27" customHeight="1"/>
+    <row r="2" ht="27" customHeight="1"/>
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2026 SAFETY ALERT LOG</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Superior Huntingdon Composites</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="10" customHeight="1"/>
+          <t>Superior Huntingdon Composites, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="8" customHeight="1"/>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -2385,6 +2397,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A6:O31"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:O2"/>
+    <mergeCell ref="A4:O4"/>
+    <mergeCell ref="A3:O3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -2396,15 +2413,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -2413,56 +2426,62 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Superior Huntingdon Composites</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Counts update automatically from the Incident Log tab</t>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>YTD TOTAL</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>RECORDABLES</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>LOSS TIME</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>HAND/FINGER</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>YTD TOTAL</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>RECORDABLES</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>LOSS TIME</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>HAND/FINGER</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
+      <c r="A7" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="B7" s="10" t="n"/>
+      <c r="C7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="9" t="n">
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="9" t="n">
         <v>10</v>
       </c>
+      <c r="H7" s="10" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A6:B6"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>